<commit_message>
fix: use AIC Normalized Supplier for accurate supplier deduplication
</commit_message>
<xml_diff>
--- a/Spend_Analysis_Output.xlsx
+++ b/Spend_Analysis_Output.xlsx
@@ -2696,7 +2696,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
@@ -2761,7 +2761,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GSD- VERPACKUNGEN</t>
+          <t>GSD VERPACKUNGEN</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -2774,7 +2774,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GROUP O</t>
+          <t xml:space="preserve">GROUP O </t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GSD- VERPACKUNGEN</t>
+          <t>GSD VERPACKUNGEN</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GROUP O</t>
+          <t xml:space="preserve">GROUP O </t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EXTENDATA SOLUTIONS LLC</t>
+          <t>EXTENDATA SOLUTIONS</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FINE ARTS DE MEXICO SA DE CV (USD)</t>
+          <t>FINE ARTS DE MEXICO SA DE CV</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BREZA PAK D.O.O.</t>
+          <t>BREZA PAK DOO</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>WELTON BIBBY &amp; BARRON LTD</t>
+          <t>WELTON BIBBY AND BARRON</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SODEXO LTD</t>
+          <t>SODEXO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -3117,7 +3117,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>THE END OF LINE D.O.O.</t>
+          <t>THE END OF LINE DOO</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MULTI SERVICES GSTJ INC</t>
+          <t>MULTI SERVICES GSTJ</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ULINE (MTY) SHIPPING SUPPLIES S DE (USD)</t>
+          <t>ULINE</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>FOKSAN D.O.O</t>
+          <t>FOKSAN DOO</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>NPB AUTOMATION AB</t>
+          <t>NPB AUTOMATION</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PROMOTORA DE MADERAS MONTERREY SA (MXN)</t>
+          <t>PROMOTORA DE MADERAS MONTERREY</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DJ LABEL SAS</t>
+          <t>DJ LABEL</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -3288,7 +3288,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>GRUPMICROS SMART SOLUTIONS, S.L.</t>
+          <t>GRUPMICROS SMART SOLUTIONS, SL</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ARDAGH METAL BEVERAGE USA</t>
+          <t>ARDAGH METAL BEVERAGE</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -3334,7 +3334,7 @@
   <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
   </cols>
@@ -3372,7 +3372,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GSD- VERPACKUNGEN</t>
+          <t>GSD VERPACKUNGEN</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -3385,7 +3385,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GROUP O</t>
+          <t xml:space="preserve">GROUP O </t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -3424,7 +3424,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EXTENDATA SOLUTIONS LLC</t>
+          <t>EXTENDATA SOLUTIONS</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -3437,7 +3437,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FINE ARTS DE MEXICO SA DE CV (USD)</t>
+          <t>FINE ARTS DE MEXICO SA DE CV</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -3489,7 +3489,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BREZA PAK D.O.O.</t>
+          <t>BREZA PAK DOO</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -3502,7 +3502,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>WELTON BIBBY &amp; BARRON LTD</t>
+          <t>WELTON BIBBY AND BARRON</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
@@ -3515,7 +3515,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SODEXO LTD</t>
+          <t>SODEXO</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -3541,7 +3541,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>THE END OF LINE D.O.O.</t>
+          <t>THE END OF LINE DOO</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -3554,7 +3554,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MULTI SERVICES GSTJ INC</t>
+          <t>MULTI SERVICES GSTJ</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
@@ -3567,7 +3567,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ULINE (MTY) SHIPPING SUPPLIES S DE (USD)</t>
+          <t>ULINE</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -3580,7 +3580,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FOKSAN D.O.O</t>
+          <t>FOKSAN DOO</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
@@ -3606,7 +3606,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NPB AUTOMATION AB</t>
+          <t>NPB AUTOMATION</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -3632,7 +3632,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PROMOTORA DE MADERAS MONTERREY SA (MXN)</t>
+          <t>PROMOTORA DE MADERAS MONTERREY</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
@@ -3645,7 +3645,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DJ LABEL SAS</t>
+          <t>DJ LABEL</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -3658,7 +3658,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GRUPMICROS SMART SOLUTIONS, S.L.</t>
+          <t>GRUPMICROS SMART SOLUTIONS, SL</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
@@ -3671,7 +3671,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ARDAGH METAL BEVERAGE USA</t>
+          <t>ARDAGH METAL BEVERAGE</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">

</xml_diff>